<commit_message>
feat(test): expand to 68 cases via DFS deep exploration
DFS additions (15 new cases):
- A011-A016: 新增页dropdown深度枚举(进货仓库16项/计税类别3项/托运责任仅2项)、商品库弹窗筛选+添加/关闭、空表单校验
- I006-I012: 料件预计领用日期筛选+搜索异常、VTable列宽拖拽/横向滚动/全选/双击无跳转/右键菜单探测
- C005-C007: 流程设置编辑→保存切换、未选择订单提示
- I008-I010: VTable列交互(列宽/滚动/全选)

Field matrix expanded from 33→43 rows with DFS depth levels (L0→L2)
Test data sheet now covers all 68 cases
</commit_message>
<xml_diff>
--- a/测试用例_托工管理_托工订单_2026-06-22.xlsx
+++ b/测试用例_托工管理_托工订单_2026-06-22.xlsx
@@ -486,11 +486,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R54"/>
+  <dimension ref="A1:R69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -499,7 +499,7 @@
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="38" customWidth="1" min="9" max="9"/>
     <col width="46" customWidth="1" min="10" max="10"/>
-    <col width="38" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
@@ -4765,6 +4765,1143 @@
       <c r="Q54" s="2" t="inlineStr"/>
       <c r="R54" s="3" t="inlineStr"/>
     </row>
+    <row r="55" ht="80" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A011</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>新增—进货仓库下拉含16个仓库可选</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>验证进货仓库下拉选项完整且可选</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>托工订单</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 进入托工订单新增页</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>1. 进入新增页
+2. 点击进货仓库下拉框
+3. 展开查看全部选项
+4. 选择「成品仓」</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>字段:进货仓库
+选项数:16
+示例:成品仓/半成品仓/1F生产仓库/2F自动化立体仓</t>
+        </is>
+      </c>
+      <c r="L55" s="3" t="inlineStr">
+        <is>
+          <t>下拉展开显示16个仓库选项
+每个选项可正常选中</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr"/>
+      <c r="N55" s="2" t="inlineStr"/>
+      <c r="O55" s="2" t="inlineStr"/>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q55" s="2" t="inlineStr"/>
+      <c r="R55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56" ht="80" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A012</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>新增—计税类别切换（不计税/应税内含/应税外加）</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>验证计税类别3个选项切换正常</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>托工订单</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 进入托工订单新增页</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>1. 点击计税类别下拉
+2. 依次切换三个选项
+3. 观察金额字段联动</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>字段:计税类别
+选项:不计税/应税内含/应税外加</t>
+        </is>
+      </c>
+      <c r="L56" s="3" t="inlineStr">
+        <is>
+          <t>3个选项均可选中并正确显示</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr"/>
+      <c r="N56" s="2" t="inlineStr"/>
+      <c r="O56" s="2" t="inlineStr"/>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="inlineStr"/>
+      <c r="R56" s="3" t="inlineStr"/>
+    </row>
+    <row r="57" ht="80" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A013</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>新增—商品库弹窗按筛选后添加商品</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>验证商品库弹窗内筛选+添加完整流程</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>托工订单</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 进入新增页
+3. 点击「从商品库选择」</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>1. 弹窗内设置货物状态和商品类型筛选
+2. 勾选商品行
+3. 点击「添加」按钮</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>货物状态:下拉选择
+商品类型:下拉选择
+操作:勾选→添加</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>商品回填到订单货物信息中
+弹窗关闭</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr"/>
+      <c r="N57" s="2" t="inlineStr"/>
+      <c r="O57" s="2" t="inlineStr"/>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q57" s="2" t="inlineStr"/>
+      <c r="R57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58" ht="80" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A014</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>新增—商品库弹窗关闭不添加</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>验证取消选择不添加商品</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>托工订单</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 商品库弹窗已打开并勾选了商品</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>1. 勾选商品后点击「关闭」按钮</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>操作:关闭</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr">
+        <is>
+          <t>弹窗关闭
+货物信息表中无新增商品行</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr"/>
+      <c r="N58" s="2" t="inlineStr"/>
+      <c r="O58" s="2" t="inlineStr"/>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q58" s="2" t="inlineStr"/>
+      <c r="R58" s="3" t="inlineStr"/>
+    </row>
+    <row r="59" ht="80" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A015</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>新增—空表单提交校验提示</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>验证全部必填项为空时提交给出明确校验</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>托工订单</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>异常测试</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 进入托工订单新增页
+3. 所有字段均为空</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>1. 不填写任何字段
+2. 直接点击「生成托工订单」按钮</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>所有字段:(空)</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>系统对必填字段给出红色校验提示
+不提交请求</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr"/>
+      <c r="N59" s="2" t="inlineStr"/>
+      <c r="O59" s="2" t="inlineStr"/>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q59" s="2" t="inlineStr"/>
+      <c r="R59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60" ht="80" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A016</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>新增—托运责任仅限供应商送货和我司提货</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>验证新增页托运责任下拉仅2个选项</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>托工订单</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 进入托工订单新增页</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>1. 点击托运责任下拉
+2. 查看全部选项
+3. 切换选择</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t>字段:托运责任
+选项:供应商送货/我司提货</t>
+        </is>
+      </c>
+      <c r="L60" s="3" t="inlineStr">
+        <is>
+          <t>仅显示2个选项
+与列表页筛选的8个选项不同（新增页为受限子集）</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr"/>
+      <c r="N60" s="2" t="inlineStr"/>
+      <c r="O60" s="2" t="inlineStr"/>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q60" s="2" t="inlineStr"/>
+      <c r="R60" s="3" t="inlineStr"/>
+    </row>
+    <row r="61" ht="80" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_I006</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>料件预计领用—领用日期范围筛选</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>验证领用表日期筛选功能</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>托工订单</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>查询</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 料件预计领用弹窗已打开</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>1. 选择领用日期范围2026-06-01至2026-06-30
+2. 点击「搜索」</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>字段:领用日期
+值:2026-06-01~2026-06-30</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="inlineStr">
+        <is>
+          <t>列表仅展示该日期范围的记录</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr"/>
+      <c r="N61" s="2" t="inlineStr"/>
+      <c r="O61" s="2" t="inlineStr"/>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q61" s="2" t="inlineStr"/>
+      <c r="R61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62" ht="80" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_I007</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>料件预计领用—搜索不存在商品</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>验证搜索不存在的商品返回空</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>托工订单</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>异常测试</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>查询</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 料件预计领用弹窗已打开</t>
+        </is>
+      </c>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>1. 输入商品识别码「NOEXIST999」
+2. 点击「搜索」</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t>搜索值:NOEXIST999</t>
+        </is>
+      </c>
+      <c r="L62" s="3" t="inlineStr">
+        <is>
+          <t>列表返回空/暂无数据</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr"/>
+      <c r="O62" s="2" t="inlineStr"/>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q62" s="2" t="inlineStr"/>
+      <c r="R62" s="3" t="inlineStr"/>
+    </row>
+    <row r="63" ht="80" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_C005</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>流程设置—编辑模式下页面切换为可编辑态</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>验证编辑按钮使页面进入编辑模式</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>托工订单</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>配置</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 进入流程设置页面</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>1. 观察只读态
+2. 点击「编辑」按钮
+3. 观察变化</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>操作:编辑</t>
+        </is>
+      </c>
+      <c r="L63" s="3" t="inlineStr">
+        <is>
+          <t>复选框可勾选
+「编辑」变为「保存」</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr"/>
+      <c r="N63" s="2" t="inlineStr"/>
+      <c r="O63" s="2" t="inlineStr"/>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q63" s="2" t="inlineStr"/>
+      <c r="R63" s="3" t="inlineStr"/>
+    </row>
+    <row r="64" ht="80" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_C006</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>流程设置—未选择订单时进入提示</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>验证未选择订单时页面提示</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>托工订单</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>配置</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 列表页未勾选任何行</t>
+        </is>
+      </c>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>1. 不选中任何行
+2. 点击「流程设置」按钮
+3. 观察页面</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>前置:未选择订单</t>
+        </is>
+      </c>
+      <c r="L64" s="3" t="inlineStr">
+        <is>
+          <t>显示「请选择托外订单!请选择一条数据」提示</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr"/>
+      <c r="N64" s="2" t="inlineStr"/>
+      <c r="O64" s="2" t="inlineStr"/>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q64" s="2" t="inlineStr"/>
+      <c r="R64" s="3" t="inlineStr"/>
+    </row>
+    <row r="65" ht="80" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_I008</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>VTable—列宽拖拽调整</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>验证VTable列宽可拖拽</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>托工订单</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>交互</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 列表页已加载</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>1. 拖拽列头边缘调整列宽
+2. 观察变化</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>操作:拖拽列头边缘</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>列宽成功调整</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr"/>
+      <c r="N65" s="2" t="inlineStr"/>
+      <c r="O65" s="2" t="inlineStr"/>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q65" s="2" t="inlineStr"/>
+      <c r="R65" s="3" t="inlineStr"/>
+    </row>
+    <row r="66" ht="80" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_I009</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>VTable—横向滚动查看全部28列</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>验证VTable横向滚动</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>托工订单</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>交互</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 列表页已加载</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>1. 向右滚动
+2. 确认最后一列可见</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>操作:横向滚动</t>
+        </is>
+      </c>
+      <c r="L66" s="3" t="inlineStr">
+        <is>
+          <t>全部28列可滚动查看
+固定列保持可见</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr"/>
+      <c r="N66" s="2" t="inlineStr"/>
+      <c r="O66" s="2" t="inlineStr"/>
+      <c r="P66" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q66" s="2" t="inlineStr"/>
+      <c r="R66" s="3" t="inlineStr"/>
+    </row>
+    <row r="67" ht="80" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_I010</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>VTable—复选框全选/取消全选</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>验证表头复选框全选功能</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>托工订单</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>选择</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 列表页已加载</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>1. 点击表头复选框全选
+2. 再点击取消</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>操作:全选→取消</t>
+        </is>
+      </c>
+      <c r="L67" s="3" t="inlineStr">
+        <is>
+          <t>全选时所有行勾选
+取消时全部取消</t>
+        </is>
+      </c>
+      <c r="M67" s="2" t="inlineStr"/>
+      <c r="N67" s="2" t="inlineStr"/>
+      <c r="O67" s="2" t="inlineStr"/>
+      <c r="P67" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q67" s="2" t="inlineStr"/>
+      <c r="R67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68" ht="80" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_I011</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>VTable—行双击无跳转（只读列表）</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>验证双击行不触发页面跳转（确认只读）</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>托工订单</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>交互</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 列表页已加载</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>1. 双击某数据行
+2. 观察URL和页面变化</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t>操作:双击行</t>
+        </is>
+      </c>
+      <c r="L68" s="3" t="inlineStr">
+        <is>
+          <t>无页面跳转
+无弹窗
+行可能高亮选中</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr"/>
+      <c r="N68" s="2" t="inlineStr"/>
+      <c r="O68" s="2" t="inlineStr"/>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q68" s="2" t="inlineStr"/>
+      <c r="R68" s="3" t="inlineStr"/>
+    </row>
+    <row r="69" ht="80" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_I012</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>VTable—右键上下文菜单（如有）</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>验证右键菜单是否存在及选项</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>托工管理</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>托工订单</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>交互</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>1. 已登录SCM系统
+2. 列表页已加载</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>1. 在某数据行上右键点击
+2. 观察是否出现菜单
+3. 点击菜单项</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>操作:右键</t>
+        </is>
+      </c>
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t>如出现菜单则记录菜单项
+如无菜单则确认无右键交互</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr"/>
+      <c r="N69" s="2" t="inlineStr"/>
+      <c r="O69" s="2" t="inlineStr"/>
+      <c r="P69" s="2" t="inlineStr">
+        <is>
+          <t>Hooplus1ce</t>
+        </is>
+      </c>
+      <c r="Q69" s="2" t="inlineStr"/>
+      <c r="R69" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4776,15 +5913,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4835,19 +5972,20 @@
           <t>托外订单号</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>text_input</t>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>TW20260622</t>
+          <t>托外订单号:TW20260622
+运算符:包含</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>≥1</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -4867,19 +6005,21 @@
           <t>订单状态</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>进行中</t>
+          <t>字段:订单状态
+运算符:等于
+值:进行中</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>~125</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -4899,19 +6039,21 @@
           <t>审批状态</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>审批通过</t>
+          <t>字段:审批状态
+运算符:等于
+值:审批通过</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>~41</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -4931,19 +6073,21 @@
           <t>审批人</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>诺贝黄小珍</t>
+          <t>字段:审批人
+运算符:等于
+值:诺贝黄小珍</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>~33</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -4963,19 +6107,21 @@
           <t>订单类型</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>委外加工</t>
+          <t>字段:订单类型
+运算符:等于
+值:委外加工</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -4995,19 +6141,21 @@
           <t>商品状态</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>待安排进货</t>
+          <t>字段:商品状态
+运算符:等于
+值:待安排进货</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>~120</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5027,19 +6175,21 @@
           <t>托运责任</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>供应商送货</t>
+          <t>字段:托运责任
+运算符:等于
+值:供应商送货</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>≥0</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5059,19 +6209,21 @@
           <t>供应商名称</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>text_input</t>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>企业名称11</t>
+          <t>字段:供应商名称
+运算符:包含
+值:企业名称11</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>~54</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5091,19 +6243,21 @@
           <t>商品名称</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>text_input</t>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>测试</t>
+          <t>字段:商品名称
+运算符:包含
+值:测试</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>≥1</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5123,19 +6277,21 @@
           <t>币别</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>人民币</t>
+          <t>字段:币别
+运算符:等于
+值:人民币</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>~138</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5147,27 +6303,29 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>单条件查询—交付日期介于</t>
+          <t>单条件查询—交付日期介于2026-06-01至2026-06-30</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>交付日期</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>date_range</t>
+          <t>交付日期介于2026-06-01至2026-06-30</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>2026-06-01~2026-06-30</t>
+          <t>字段:交付日期
+运算符:介于
+值:2026-06-01~2026-06-30</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>≥1</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5187,19 +6345,21 @@
           <t>托工负责人</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>text_input</t>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>黄小珍</t>
+          <t>字段:托工负责人
+运算符:包含
+值:黄小珍</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>≥1</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5211,7 +6371,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>组合查询—订单状态+商品状态(2条件)</t>
+          <t>组合查询—订单状态+商品状态（2条件AND）</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -5219,19 +6379,20 @@
           <t>订单状态+商品状态</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>multi</t>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>进行中 + 待安排进货</t>
+          <t>条件1 订单状态=进行中
+条件2 商品状态=待安排进货</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>待验证</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5243,27 +6404,28 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>组合查询—供应商名称+商品名称(2条件)</t>
+          <t>组合查询—供应商名称+商品名称（2条件AND）</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>供应商+商品名称</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>multi</t>
+          <t>供应商名称+商品名称</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>企业名称11 + 测试</t>
+          <t>条件1 供应商名称包含=企业名称11
+条件2 商品名称包含=测试</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>待验证</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5275,7 +6437,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>组合查询—3条件AND</t>
+          <t>组合查询—订单状态+审批状态+交付日期（3条件AND）</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -5283,19 +6445,21 @@
           <t>订单状态+审批状态+交付日期</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>multi</t>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>进行中 + 审批通过 + 2026-06</t>
+          <t>条件1 订单状态=进行中
+条件2 审批状态=审批通过
+条件3 交付日期=2026-06-01~2026-06-30</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>待验证</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5307,7 +6471,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>组合查询—4条件AND</t>
+          <t>组合查询—商品状态+托运责任+币别+托工负责人（4条件AND）</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -5315,19 +6479,22 @@
           <t>商品状态+托运责任+币别+托工负责人</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>multi</t>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>待安排进货+供应商送货+人民币+诺贝</t>
+          <t>商品状态=待安排进货
+托运责任=供应商送货
+币别=人民币
+托工负责人包含=诺贝</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>待验证</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -5339,7 +6506,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>边界值—采购数量等于0.1</t>
+          <t>边界值—采购数量等于最小值0.1</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -5347,19 +6514,21 @@
           <t>采购数量</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>text_input</t>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>边界值测试</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>字段:采购数量
+运算符:等于
+值:0.1</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>≥0</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -5371,7 +6540,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>边界值—采购数量等于9570</t>
+          <t>边界值—采购数量等于最大值9570</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -5379,19 +6548,21 @@
           <t>采购数量</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>text_input</t>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>边界值测试</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>9570</t>
+          <t>字段:采购数量
+运算符:等于
+值:9570</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>≥0</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -5403,7 +6574,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>边界值—金额等于0</t>
+          <t>边界值—金额等于最小值0</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -5411,19 +6582,21 @@
           <t>金额</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>text_input</t>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>边界值测试</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>字段:金额
+运算符:等于
+值:0</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>≥0</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -5435,7 +6608,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>边界值—金额等于2000</t>
+          <t>边界值—金额等于最大值2000</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -5443,19 +6616,21 @@
           <t>金额</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>text_input</t>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>边界值测试</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>字段:金额
+运算符:等于
+值:2000</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>≥0</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -5467,27 +6642,29 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>异常—不存在的订单号</t>
+          <t>异常查询—不存在的托外订单号</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>托外订单号</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>text_input</t>
+          <t>不存在的托外订单号</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>异常测试</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>NOTEXIST999999</t>
+          <t>字段:托外订单号
+运算符:包含
+值:NOTEXIST999999</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -5499,27 +6676,29 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>异常—不存在的供应商</t>
+          <t>异常查询—不存在的供应商名称</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>供应商名称</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>text_input</t>
+          <t>不存在的供应商名称</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>异常测试</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>火星供应商XYZ</t>
+          <t>字段:供应商名称
+运算符:包含
+值:火星供应商XYZ</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -5531,27 +6710,30 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>异常—日期范围非法</t>
+          <t>异常查询—交付日期结束值早于起始值</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>交付日期</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>date_range</t>
+          <t>交付日期结束值早于起始值</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>异常测试</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>2026-12-31~2026-01-01</t>
+          <t>字段:交付日期
+运算符:介于
+起始值:2026-12-31
+结束值:2026-01-01</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>0或报错</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -5568,22 +6750,23 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>reset</t>
+          <t>重置筛选条件</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>重置前条件: 订单状态=已完成
+重置后条件: 全部清空</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5595,7 +6778,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>组合查询—3条件AND(下拉)</t>
+          <t>组合查询—订单状态+审批人+商品状态（3条件AND）</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -5603,19 +6786,21 @@
           <t>订单状态+审批人+商品状态</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>multi</t>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>进行中+诺贝黄小珍+待安排进货</t>
+          <t>条件1 订单状态=进行中
+条件2 审批人=诺贝黄小珍
+条件3 商品状态=待安排进货</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>待验证</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5627,27 +6812,29 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>日期—创建时间介于</t>
+          <t>日期筛选—创建时间介于2026-06-20至2026-06-22</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>创建时间</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>date_range</t>
+          <t>创建时间介于2026-06-20至2026-06-22</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20~2026-06-22</t>
+          <t>字段:创建时间
+运算符:介于
+值:2026-06-20~2026-06-22</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>≥1</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5659,27 +6846,29 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>日期—完成时间等于当天</t>
+          <t>日期筛选—完成时间介于2026-06-22当天</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>完成时间</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>date_range</t>
+          <t>完成时间介于2026-06-22当天</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>2026-06-22~2026-06-22</t>
+          <t>字段:完成时间
+运算符:介于
+值:2026-06-22~2026-06-22</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>≥1</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5691,27 +6880,29 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>订单状态=已终止</t>
+          <t>订单状态等于「已终止」</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>订单状态</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+          <t>订单状态等于「已终止」</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>已终止</t>
+          <t>字段:订单状态
+运算符:等于
+值:已终止</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>~3</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -5723,27 +6914,32 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>新增—完整填写提交</t>
+          <t>新增—完整填写基本信息后生成托工订单成功</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>供应商+商品+附件</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>form</t>
+          <t>完整填写基本信息后生成托工订单成功</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>所有必填项</t>
+          <t>供应商名称:企业名称11
+供应商编码:供应商编码0011
+托运责任:供应商送货
+订单类型:委外加工
+订单币别:人民币
+托</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>1条新增</t>
+          <t>P0</t>
         </is>
       </c>
     </row>
@@ -5755,27 +6951,28 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>新增—供应商为空校验</t>
+          <t>新增—供应商名称为空时提交校验拦截</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>供应商名称</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>form_validation</t>
+          <t>供应商名称为空时提交校验拦截</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>(空)</t>
+          <t>供应商名称: (空)
+其他字段:已填</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>校验拦截</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5787,27 +6984,29 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>新增—托运责任切换</t>
+          <t>新增—托运责任切换选择「客户提货」</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>托运责任</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+          <t>托运责任切换选择「客户提货」</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>客户提货</t>
+          <t>字段:托运责任
+原值:供应商送货
+新值:客户提货</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>切换成功</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5819,27 +7018,28 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>新增—币别切换美元</t>
+          <t>新增—币别切换到「美元」后单价金额联动</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>币别</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>select_dropdown</t>
+          <t>币别切换到「美元」后单价金额联动</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>美元</t>
+          <t>币别:美元
+商品单价:10</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>金额联动</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -5851,27 +7051,28 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>新增—从商品库选择</t>
+          <t>新增—从商品库选择商品</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>从商品库选择按钮</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>button_modal</t>
+          <t>从商品库选择商品</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>搜索:测试</t>
+          <t>操作:从商品库选择
+搜索关键词:测试</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>选择回填</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -5883,27 +7084,28 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>新增—附件上传PDF</t>
+          <t>新增—附件上传PDF文件</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>附件上传</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>file_upload</t>
+          <t>附件上传PDF文件</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>PDF ≤5MB</t>
+          <t>文件类型:pdf
+文件大小:≤5MB</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>上传成功</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -5915,27 +7117,28 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>新增—附件超5个限制</t>
+          <t>新增—附件上传超过5个文件时提示限制</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>附件上传</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>boundary</t>
+          <t>附件上传超过5个文件时提示限制</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>边界值测试</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>6个文件</t>
+          <t>已上传文件数:5
+第6个文件:任意</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>提示限制</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -5947,27 +7150,27 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>新增—附件超5MB限制</t>
+          <t>新增—附件上传超过5MB文件时提示限制</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>附件上传</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>boundary</t>
+          <t>附件上传超过5MB文件时提示限制</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>边界值测试</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>&gt;5MB文件</t>
+          <t>文件大小:&gt;5MB</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>提示限制</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -5979,27 +7182,27 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>新增—返回按钮</t>
+          <t>新增—点击「返回」按钮回到列表</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>返回</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>button_nav</t>
+          <t>点击「返回」按钮回到列表</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>操作:返回</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>回到列表</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -6011,27 +7214,27 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>新增—用料清单tab切换</t>
+          <t>新增—用料清单tab切换查看</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>用料清单</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>tab_switch</t>
+          <t>用料清单tab切换查看</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>操作:切换tab</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>切换成功</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -6043,27 +7246,27 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>流程设置—进入页面</t>
+          <t>流程设置—进入流程发起规则设置页面</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>流程设置</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>button_nav</t>
+          <t>进入流程发起规则设置页面</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>操作:流程设置</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>页面加载</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -6075,27 +7278,28 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>流程设置—勾选触发字段</t>
+          <t>流程设置—勾选/取消订单创建触发字段</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>复选框</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>checkbox</t>
+          <t>勾选/取消订单创建触发字段</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>供应商名称</t>
+          <t>选中字段:供应商名称
+取消字段:托工单号</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>勾选成功</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -6107,27 +7311,28 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>流程设置—切换流程类型</t>
+          <t>流程设置—切换到「托工订单结案」流程类型</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>流程类型</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>radio</t>
+          <t>切换到「托工订单结案」流程类型</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>托工订单结案</t>
+          <t>原选择:新建托工订单
+新选择:托工订单结案</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>切换成功</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -6139,27 +7344,27 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>流程设置—编辑保存</t>
+          <t>流程设置—点击「编辑」进入编辑模式后保存</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>编辑按钮</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>button_edit</t>
+          <t>点击「编辑」进入编辑模式后保存</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>修改字段→保存</t>
+          <t>操作:编辑→修改→保存</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>保存成功</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -6176,22 +7381,24 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>订单状态列头</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>vtable_filter</t>
+          <t>按值筛选</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>勾选:进行中</t>
+          <t>列:订单状态
+筛选方式:按值筛选
+选中值:进行中</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>筛选有效</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -6203,27 +7410,30 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>VTable列头筛选—按条件筛选</t>
+          <t>VTable列头筛选—按条件筛选（数字列）</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>采购数量列头</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>vtable_filter</t>
+          <t>按条件筛选</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>条件:大于 100</t>
+          <t>列:采购数量
+筛选方式:按条件筛选
+条件:大于
+值:100</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>筛选有效</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -6235,27 +7445,28 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>料件预计领用—搜索</t>
+          <t>料件预计领用—打开弹窗并搜索商品</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>商品识别码</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>modal_search</t>
+          <t>打开弹窗并搜索商品</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>搜索商品</t>
+          <t>操作:料件预计领用
+搜索字段:商品识别码</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>弹窗数据</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -6267,27 +7478,28 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>料件预计领用—重置</t>
+          <t>料件预计领用—重置搜索条件</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>重置按钮</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>modal_reset</t>
+          <t>重置搜索条件</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>重置前搜索:商品识别码=XXX
+重置后:搜索条件清空</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>恢复全部</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -6299,27 +7511,27 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>VTable复选框—行选择</t>
+          <t>VTable复选框行选择—勾选后工具栏状态变化</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>复选框列</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>checkbox_row</t>
+          <t>勾选后工具栏状态变化</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>勾选多行</t>
+          <t>操作:勾选复选框</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>选择高亮</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -6336,22 +7548,23 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>导出</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>export</t>
+          <t>导出全部数据</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>无筛选</t>
+          <t>筛选条件:无（全部数据）
+操作:导出</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>P1</t>
         </is>
       </c>
     </row>
@@ -6363,27 +7576,29 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>筛选后导出</t>
+          <t>筛选后导出数据</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>导出</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>export</t>
+          <t>筛选后导出数据</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>订单状态=已完成</t>
+          <t>筛选条件:订单状态=已完成
+预期筛选结果:约12条
+操作:导出</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>~12</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -6395,27 +7610,27 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>打印功能</t>
+          <t>打印功能—触发浏览器打印</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>打印</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>print</t>
+          <t>触发浏览器打印</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>操作:打印</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>浏览器打印</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -6427,27 +7642,28 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>多标签页切换</t>
+          <t>多标签页切换—列表↔新增tab</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>标签页</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>tab_switch</t>
+          <t>列表↔新增tab</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>兼容性测试</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>列表↔新增</t>
+          <t>tab1:托工订单(已筛选)
+tab2:托工订单新增(已填部分)</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>状态保持</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -6459,27 +7675,27 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>页面刷新</t>
+          <t>列表页VTable数据刷新</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>刷新</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>refresh</t>
+          <t>列表页VTable数据刷新</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>操作:页面刷新</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>数据重载</t>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -6496,22 +7712,509 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>展开▼/收起▲</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>toggle</t>
+          <t>展开/收起筛选区域</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>操作:展开▼ → 收起▲</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>流畅切换</t>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A011</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>新增—进货仓库下拉含16个仓库可选</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>进货仓库下拉含16个仓库可选</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>字段:进货仓库
+选项数:16
+示例:成品仓/半成品仓/1F生产仓库/2F自动化立体仓</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A012</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>新增—计税类别切换（不计税/应税内含/应税外加）</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>计税类别切换</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>字段:计税类别
+选项:不计税/应税内含/应税外加</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A013</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>新增—商品库弹窗按筛选后添加商品</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>商品库弹窗按筛选后添加商品</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>货物状态:下拉选择
+商品类型:下拉选择
+操作:勾选→添加</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A014</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>新增—商品库弹窗关闭不添加</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>商品库弹窗关闭不添加</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>操作:关闭</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A015</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>新增—空表单提交校验提示</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>空表单提交校验提示</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>异常测试</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>所有字段:(空)</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_A016</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>新增—托运责任仅限供应商送货和我司提货</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>托运责任仅限供应商送货和我司提货</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>字段:托运责任
+选项:供应商送货/我司提货</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_I006</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>料件预计领用—领用日期范围筛选</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>领用日期范围筛选</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>字段:领用日期
+值:2026-06-01~2026-06-30</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_I007</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>料件预计领用—搜索不存在商品</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>搜索不存在商品</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>异常测试</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>搜索值:NOEXIST999</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_C005</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>流程设置—编辑模式下页面切换为可编辑态</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>编辑模式下页面切换为可编辑态</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>操作:编辑</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_C006</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>流程设置—未选择订单时进入提示</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>未选择订单时进入提示</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>前置:未选择订单</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_I008</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>VTable—列宽拖拽调整</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>列宽拖拽调整</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>操作:拖拽列头边缘</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_I009</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>VTable—横向滚动查看全部28列</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>横向滚动查看全部28列</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>操作:横向滚动</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_I010</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>VTable—复选框全选/取消全选</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>复选框全选/取消全选</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>操作:全选→取消</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_I011</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>VTable—行双击无跳转（只读列表）</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>行双击无跳转</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>操作:双击行</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>NB_TGDD_I012</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>VTable—右键上下文菜单（如有）</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>右键上下文菜单</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>操作:右键</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -6526,15 +8229,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6560,12 +8263,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>运算符/交互方式</t>
+          <t>交互方式/选项</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>枚举选项(下拉字段)</t>
+          <t>DFS深度</t>
         </is>
       </c>
     </row>
@@ -6577,7 +8280,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>筛选区-文本</t>
+          <t>筛选区</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -6597,7 +8300,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>L0</t>
         </is>
       </c>
     </row>
@@ -6609,7 +8312,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>筛选区-下拉</t>
+          <t>筛选区</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -6624,12 +8327,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>等于/不等于</t>
+          <t>8选项(待报价→已终止)</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>待报价/待接单/已接单/待确认/进行中/待验收/已完成/已终止</t>
+          <t>L0</t>
         </is>
       </c>
     </row>
@@ -6641,7 +8344,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>筛选区-下拉</t>
+          <t>筛选区</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -6656,12 +8359,12 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>等于/不等于</t>
+          <t>审批中/审批通过/审批驳回</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>审批中/审批通过/审批驳回</t>
+          <t>L0</t>
         </is>
       </c>
     </row>
@@ -6673,7 +8376,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>筛选区-下拉</t>
+          <t>筛选区</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -6688,12 +8391,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>等于/不等于</t>
+          <t>58人</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>58人（诺贝黄小珍等）</t>
+          <t>L0</t>
         </is>
       </c>
     </row>
@@ -6705,7 +8408,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>筛选区-下拉</t>
+          <t>筛选区</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -6720,12 +8423,12 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>包含/等于</t>
+          <t>普通采购/委外加工</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>普通采购/委外加工</t>
+          <t>L0</t>
         </is>
       </c>
     </row>
@@ -6737,7 +8440,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>筛选区-下拉</t>
+          <t>筛选区</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -6752,12 +8455,12 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>等于/不等于</t>
+          <t>6选项(待安排进货→已取消)</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>待安排进货/部分安排进货/待进货/部分进货/全部进货/已取消</t>
+          <t>L0</t>
         </is>
       </c>
     </row>
@@ -6769,7 +8472,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>筛选区-下拉</t>
+          <t>筛选区</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -6784,12 +8487,12 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>等于/不等于</t>
+          <t>8选项</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>客户提货/我司送货/我司提货/供应商送货/出货仓库送货/货仓库提货/供应商提货/客户送返</t>
+          <t>L0</t>
         </is>
       </c>
     </row>
@@ -6801,7 +8504,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>筛选区-下拉</t>
+          <t>筛选区</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -6816,12 +8519,12 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>等于/不等于</t>
+          <t>11选项(成品→外包)</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>成品/物料/半成品/商品/制成品/原料/下脚品/包装物/人工/费用/外包</t>
+          <t>L0</t>
         </is>
       </c>
     </row>
@@ -6833,7 +8536,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>筛选区-下拉</t>
+          <t>筛选区</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -6848,12 +8551,12 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>等于/不等于</t>
+          <t>22种货币</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>22种（人民币/美元/欧元等）</t>
+          <t>L0</t>
         </is>
       </c>
     </row>
@@ -6865,27 +8568,27 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>筛选区-下拉</t>
+          <t>筛选区</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>单位</t>
+          <t>交付日期等4个</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>select_dropdown</t>
+          <t>date_range</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>包含/等于</t>
+          <t>介于</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>个/具</t>
+          <t>L0</t>
         </is>
       </c>
     </row>
@@ -6897,27 +8600,27 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>筛选区-下拉</t>
+          <t>工具栏</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>交付地点</t>
+          <t>新增</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>select_dropdown</t>
+          <t>button_nav</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>包含/等于</t>
+          <t>打开新tab(laborOrderDetail)</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>中山/中山世通医疗</t>
+          <t>L1→新增页</t>
         </is>
       </c>
     </row>
@@ -6929,27 +8632,27 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>筛选区-下拉</t>
+          <t>工具栏</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>托工负责人</t>
+          <t>设置</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>select_dropdown</t>
+          <t>button_vtable</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>包含/等于</t>
+          <t>VTable列配置(Canvas级)</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>58人</t>
+          <t>L1</t>
         </is>
       </c>
     </row>
@@ -6961,27 +8664,27 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>筛选区-数值</t>
+          <t>工具栏</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>采购数量/已缴库数量/未交数量/单价/金额</t>
+          <t>导出</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>text_input</t>
+          <t>button_export</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>等于/不等于</t>
+          <t>导出Excel</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>0.1~9570 / 0~2000</t>
+          <t>L1</t>
         </is>
       </c>
     </row>
@@ -6993,27 +8696,27 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>筛选区-日期</t>
+          <t>工具栏</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>交付日期/需交付日期/完成时间/创建时间</t>
+          <t>打印</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>date_range</t>
+          <t>button_print</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>介于</t>
+          <t>浏览器打印</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>L1</t>
         </is>
       </c>
     </row>
@@ -7030,22 +8733,22 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>新增</t>
+          <t>料件预计领用</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>button_nav</t>
+          <t>button_modal</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>打开新增tab(laborOrderDetail)</t>
+          <t>弹出领用表弹窗</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>L1→弹窗</t>
         </is>
       </c>
     </row>
@@ -7062,22 +8765,22 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>设置</t>
+          <t>流程设置</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>button_vtable</t>
+          <t>button_nav</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>VTable列设置(Canvas级)</t>
+          <t>跳转/flowSet</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>L1→配置页</t>
         </is>
       </c>
     </row>
@@ -7089,27 +8792,27 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>工具栏</t>
+          <t>VTable</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>导出</t>
+          <t>复选框列</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>button_export</t>
+          <t>checkbox</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>导出Excel</t>
+          <t>行选择/全选</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>L1</t>
         </is>
       </c>
     </row>
@@ -7121,27 +8824,27 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>工具栏</t>
+          <t>VTable</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>打印</t>
+          <t>列头点击</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>button_print</t>
+          <t>vtable_filter</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>浏览器打印</t>
+          <t>按值筛选/按条件筛选</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>L1</t>
         </is>
       </c>
     </row>
@@ -7153,27 +8856,27 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>工具栏</t>
+          <t>VTable</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>料件预计领用</t>
+          <t>列头拖拽</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>button_modal</t>
+          <t>drag</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>弹出料件预计领用表</t>
+          <t>列宽调整</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>L1</t>
         </is>
       </c>
     </row>
@@ -7185,98 +8888,98 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>工具栏</t>
+          <t>VTable</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>流程设置</t>
+          <t>横向滚动</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>button_nav</t>
+          <t>scroll</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>跳转/flowSet</t>
+          <t>查看全部28列</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>L1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>托工订单列表</t>
+          <t>新增页</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>VTable交互</t>
+          <t>基本信息</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>复选框列</t>
+          <t>供应商名称</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>checkbox</t>
+          <t>select_dropdown</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>行选择</t>
+          <t>8个供应商</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>L1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>托工订单列表</t>
+          <t>新增页</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>VTable交互</t>
+          <t>基本信息</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>列头点击</t>
+          <t>供应商编码</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>vtable_filter</t>
+          <t>select_dropdown</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>按值筛选/按条件筛选</t>
+          <t>8个编码(随供应商联动)</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>L1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>托工订单新增</t>
+          <t>新增页</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -7286,29 +8989,29 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>供应商名称</t>
+          <t>计税类别</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>text_input+select</t>
+          <t>select_dropdown</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>输入+下拉搜索</t>
+          <t>不计税/应税内含/应税外加</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>9家供应商</t>
+          <t>L1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>托工订单新增</t>
+          <t>新增页</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -7328,19 +9031,19 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>等于</t>
+          <t>供应商送货/我司提货(仅2项)</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>8选项</t>
+          <t>L1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>托工订单新增</t>
+          <t>新增页</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -7350,7 +9053,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>订单类型</t>
+          <t>进货仓库</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -7360,19 +9063,19 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>等于</t>
+          <t>16个仓库</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>普通采购/委外加工</t>
+          <t>L1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>托工订单新增</t>
+          <t>新增页</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -7382,7 +9085,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>订单币别</t>
+          <t>订单类型</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -7392,51 +9095,51 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>等于</t>
+          <t>普通采购/委外加工(注意:可能误显仓库名)</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>22种</t>
+          <t>L1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>托工订单新增</t>
+          <t>新增页</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>货物信息</t>
+          <t>基本信息</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>委外商品/用料清单</t>
+          <t>订单币别</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>tab</t>
+          <t>select_dropdown</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>tab切换</t>
+          <t>默认为人民币</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>L1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>托工订单新增</t>
+          <t>新增页</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -7456,172 +9159,492 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>商品选择弹窗</t>
+          <t>打开商品库弹窗</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>L1→L2弹窗</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>托工订单新增</t>
+          <t>新增页→商品库弹窗</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>附件列表</t>
+          <t>弹窗</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>文件上传</t>
+          <t>货物状态</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>file_upload</t>
+          <t>select_dropdown</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>拖拽/点击</t>
+          <t>筛选字段</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>≤5文件×≤5MB,14种格式</t>
+          <t>L2</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>托工订单新增</t>
+          <t>新增页→商品库弹窗</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>页面按钮</t>
+          <t>弹窗</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>返回/列表/生成托工订单</t>
+          <t>商品类型</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>select_dropdown</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>导航/提交</t>
+          <t>筛选字段</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>L2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>流程设置</t>
+          <t>新增页→商品库弹窗</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>页面</t>
+          <t>弹窗</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>流程类型</t>
+          <t>VTable</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>radio</t>
+          <t>vtable_checkbox</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>新建托工订单/托工订单结案</t>
+          <t>勾选商品行</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>L2</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>流程设置</t>
+          <t>新增页→商品库弹窗</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>页面</t>
+          <t>弹窗</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>触发字段</t>
+          <t>添加/关闭</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>checkbox</t>
+          <t>button</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>勾选/取消</t>
+          <t>确认添加或取消</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>27个字段</t>
+          <t>L2</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>流程设置</t>
+          <t>新增页</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
+          <t>附件列表</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>文件上传</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>file_upload</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>拖拽/点击;≤5文件×≤5MB;14种格式</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>新增页</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
           <t>页面按钮</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>编辑/返回</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>生成托工订单</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>button_submit</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>提交创建</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>新增页</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>页面按钮</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>返回/列表</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>button_nav</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>回到列表</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>料件预计领用弹窗</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>弹窗</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>商品识别码/名称</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>text_input</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>搜索</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>料件预计领用弹窗</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>弹窗</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>领用日期</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>date_range</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>日期范围筛选</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>料件预计领用弹窗</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>弹窗</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>HTML表格</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>table_checkbox</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>15列物料数据+复选框</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>料件预计领用弹窗</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>弹窗按钮</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>搜索/重置</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>button</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>编辑模式/导航</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>查询/清空</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>流程设置页</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>页面</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>流程类型</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>radio</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>新建托工订单/托工订单结案</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>流程设置页</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>页面</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>触发字段</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>checkbox</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>27个字段(供应商/托工单号等)</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>流程设置页</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>页面按钮</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>编辑/保存</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>button_toggle</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>切换只读/编辑模式</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>流程设置页</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>页面按钮</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>返回</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>button_nav</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>回到列表</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
         </is>
       </c>
     </row>

</xml_diff>